<commit_message>
Nouveau système RSVP : QR code unique, recherche par nom, hébergement
- rsvp.html : page publique avec recherche par nom, formulaire présence/hébergement (75€/2 nuits), page de confirmation stylée
- server.py : endpoints /api/rsvp/search et /api/rsvp/submit, champ hébergement + rsvpSubmittedAt dans le modèle invité
- organisation.html + script.js : case hébergement par invité, stats hébergement (foyers, personnes, revenus)
- Excel : colonne hébergement dans la feuille Invités RSVP, stats hébergement dans le récapitulatif

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/budget_mariage.xlsx
+++ b/budget_mariage.xlsx
@@ -8,11 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Budget Mariage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Invites RSVP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Invités RSVP" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Budget Mariage'!$A$14:$C$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Invites RSVP'!$A$11:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Budget Mariage'!$A$14:$F$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Invités RSVP'!$A$11:$F$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -88,7 +88,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E6"/>
+        <fgColor rgb="00E8F6ED"/>
       </patternFill>
     </fill>
   </fills>
@@ -533,12 +533,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -551,11 +554,11 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Mise a jour</t>
+          <t>Mise à jour</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46086.68590770834</v>
+        <v>46133.51778204861</v>
       </c>
     </row>
     <row r="4">
@@ -571,11 +574,11 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Depenses engagees</t>
+          <t>Dépenses engagées</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>22200</v>
+        <v>17849</v>
       </c>
     </row>
     <row r="6">
@@ -585,23 +588,23 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>2800</v>
+        <v>7151</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Part du budget utilisee</t>
+          <t>Part du budget utilisée</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>0.888</v>
+        <v>0.71396</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Invites prevus</t>
+          <t>Invités prévus</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
@@ -611,7 +614,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Adultes prevus</t>
+          <t>Adultes prévus</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
@@ -621,35 +624,50 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Cout moyen par invite</t>
+          <t>Coût moyen par invité</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>148</v>
+        <v>118.9933333333333</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Cout moyen par adulte</t>
+          <t>Coût moyen par adulte</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>201.8181818181818</v>
+        <v>162.2636363636364</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Poste de depense</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Montant</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Montant total prévu</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Déjà payé</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Reste à payer</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Part du budget</t>
         </is>
@@ -658,122 +676,186 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Les Domaines de Gaston (Les Andelys)</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>8000</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>0.32</v>
+          <t>Lieux</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Les domaines de Gaston</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>7300</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>2100</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>5200</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.292</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Traiteur</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>8000</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>0.32</v>
+          <t>Photo/Vidéo</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Photographe</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>2400</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>720</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>1680</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0.096</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Photographe</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>0.06</v>
+          <t>Traiteurs</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Gastron'Home</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>5529</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>1658</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>3871</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0.22116</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Faire-Part</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>400</v>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>0.016</v>
+          <t>Traiteurs</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Food-truck pizza</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>1120</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>336</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>784</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0.0448</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Fleuriste</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>0.04</v>
+          <t>Traiteurs</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Food-truck sucré</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>280</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0.016</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>DJ</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>1300</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>0.052</v>
+          <t>Décoration</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Lettres géantes</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Décoration</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>0.06</v>
+          <t>Traiteurs</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Serveurs</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0.04</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Église de Gisors</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>500</v>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="10" t="n">
-        <v>22200</v>
-      </c>
-      <c r="C23" s="11" t="n">
-        <v>0.888</v>
+      <c r="C22" s="10" t="n">
+        <v>17849</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>0.71396</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A14:C23"/>
+  <autoFilter ref="A14:F22"/>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
@@ -787,7 +869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -801,44 +883,44 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Liste des invites et RSVP</t>
+          <t>Liste des invités et RSVP</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Foyers invites</t>
+          <t>Foyers invités</t>
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Personnes invitees</t>
+          <t>Personnes invitées</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Personnes confirmees</t>
+          <t>Personnes confirmées</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Personnes declinees</t>
+          <t>Personnes refusées</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -852,7 +934,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -862,7 +944,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -913,7 +995,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>En attente</t>
+          <t>Confirme</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -928,25 +1010,56 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>DURAND Nicolas</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Confirme</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Vin d'honneur + repas</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8000/rsvp?token=g_xpf62papwyt00mtm</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>TOTAL PERSONNES</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="16" t="n">
-        <v>0</v>
+      <c r="C14" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A11:F13"/>
+  <autoFilter ref="A11:F14"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>